<commit_message>
add shipvault unit-record url as second ref wherever the page renders blank; companion batch for existing backend cells
</commit_message>
<xml_diff>
--- a/batches/2026-09-17_0431ET_discovery_since_jun_2026/lng_carrier_candidate_vessels.xlsx
+++ b/batches/2026-09-17_0431ET_discovery_since_jun_2026/lng_carrier_candidate_vessels.xlsx
@@ -1872,7 +1872,7 @@
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>https://www.shipvault.com/ships/502918</t>
+          <t>https://www.shipvault.com/ships/502918, https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/502918</t>
         </is>
       </c>
       <c r="H8" s="7" t="inlineStr">
@@ -1891,7 +1891,7 @@
       </c>
       <c r="N8" s="7" t="inlineStr">
         <is>
-          <t>https://www.shipvault.com/ships/502918</t>
+          <t>https://www.shipvault.com/ships/502918, https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/502918</t>
         </is>
       </c>
       <c r="O8" s="7" t="inlineStr">
@@ -2040,7 +2040,7 @@
       </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
-          <t>https://www.shipvault.com/ships/502919</t>
+          <t>https://www.shipvault.com/ships/502919, https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/502919</t>
         </is>
       </c>
       <c r="H9" s="7" t="inlineStr">
@@ -2059,7 +2059,7 @@
       </c>
       <c r="N9" s="7" t="inlineStr">
         <is>
-          <t>https://www.shipvault.com/ships/502919</t>
+          <t>https://www.shipvault.com/ships/502919, https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/502919</t>
         </is>
       </c>
       <c r="O9" s="7" t="inlineStr">
@@ -2208,7 +2208,7 @@
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>https://www.shipvault.com/ships/502920</t>
+          <t>https://www.shipvault.com/ships/502920, https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/502920</t>
         </is>
       </c>
       <c r="H10" s="7" t="inlineStr">
@@ -2227,7 +2227,7 @@
       </c>
       <c r="N10" s="7" t="inlineStr">
         <is>
-          <t>https://www.shipvault.com/ships/502920</t>
+          <t>https://www.shipvault.com/ships/502920, https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/502920</t>
         </is>
       </c>
       <c r="O10" s="7" t="inlineStr">
@@ -2376,7 +2376,7 @@
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
-          <t>https://www.shipvault.com/ships/502921</t>
+          <t>https://www.shipvault.com/ships/502921, https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/502921</t>
         </is>
       </c>
       <c r="H11" s="7" t="inlineStr">
@@ -2395,7 +2395,7 @@
       </c>
       <c r="N11" s="7" t="inlineStr">
         <is>
-          <t>https://www.shipvault.com/ships/502921</t>
+          <t>https://www.shipvault.com/ships/502921, https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/502921</t>
         </is>
       </c>
       <c r="O11" s="7" t="inlineStr">
@@ -2544,7 +2544,7 @@
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
-          <t>https://www.shipvault.com/ships/503416</t>
+          <t>https://www.shipvault.com/ships/503416, https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/503416</t>
         </is>
       </c>
       <c r="H12" s="7" t="inlineStr">
@@ -2563,7 +2563,7 @@
       </c>
       <c r="N12" s="7" t="inlineStr">
         <is>
-          <t>https://www.shipvault.com/ships/503416</t>
+          <t>https://www.shipvault.com/ships/503416, https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/503416</t>
         </is>
       </c>
       <c r="O12" s="7" t="inlineStr">
@@ -2712,7 +2712,7 @@
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
-          <t>https://www.shipvault.com/ships/503417</t>
+          <t>https://www.shipvault.com/ships/503417, https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/503417</t>
         </is>
       </c>
       <c r="H13" s="7" t="inlineStr">
@@ -2731,7 +2731,7 @@
       </c>
       <c r="N13" s="7" t="inlineStr">
         <is>
-          <t>https://www.shipvault.com/ships/503417</t>
+          <t>https://www.shipvault.com/ships/503417, https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/503417</t>
         </is>
       </c>
       <c r="O13" s="7" t="inlineStr">
@@ -3086,7 +3086,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>https://www.worldoil.com/news/2026/7/10/adnoc-l-s-orders-four-lng-carriers-to-expand-global-shipping-fleet/, https://gasprocessingnews.com/news/2026/07/adnoc-ls-expands-lng-fleet-with-order-for-four-new-carriers/, http://www.chinashipbuild.com/ship.aspx?pklujyukkpp4JsCcXanmkhTk8Pl4EN, https://www.shipvault.com/ships/502918</t>
+          <t>https://www.worldoil.com/news/2026/7/10/adnoc-l-s-orders-four-lng-carriers-to-expand-global-shipping-fleet/, https://gasprocessingnews.com/news/2026/07/adnoc-ls-expands-lng-fleet-with-order-for-four-new-carriers/, http://www.chinashipbuild.com/ship.aspx?pklujyukkpp4JsCcXanmkhTk8Pl4EN, https://www.shipvault.com/ships/502918, https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/502918</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -3113,7 +3113,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>https://www.worldoil.com/news/2026/7/10/adnoc-l-s-orders-four-lng-carriers-to-expand-global-shipping-fleet/, https://gasprocessingnews.com/news/2026/07/adnoc-ls-expands-lng-fleet-with-order-for-four-new-carriers/, http://www.chinashipbuild.com/ship.aspx?pklujyukkpp4JsCcXanmkhTk8Pl4EN, https://www.shipvault.com/ships/502919</t>
+          <t>https://www.worldoil.com/news/2026/7/10/adnoc-l-s-orders-four-lng-carriers-to-expand-global-shipping-fleet/, https://gasprocessingnews.com/news/2026/07/adnoc-ls-expands-lng-fleet-with-order-for-four-new-carriers/, http://www.chinashipbuild.com/ship.aspx?pklujyukkpp4JsCcXanmkhTk8Pl4EN, https://www.shipvault.com/ships/502919, https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/502919</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -3140,7 +3140,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>https://www.worldoil.com/news/2026/7/10/adnoc-l-s-orders-four-lng-carriers-to-expand-global-shipping-fleet/, https://gasprocessingnews.com/news/2026/07/adnoc-ls-expands-lng-fleet-with-order-for-four-new-carriers/, http://www.chinashipbuild.com/ship.aspx?pklujyukkpp4JsCcXanmkhTk8Pl4EN, https://www.shipvault.com/ships/502920</t>
+          <t>https://www.worldoil.com/news/2026/7/10/adnoc-l-s-orders-four-lng-carriers-to-expand-global-shipping-fleet/, https://gasprocessingnews.com/news/2026/07/adnoc-ls-expands-lng-fleet-with-order-for-four-new-carriers/, http://www.chinashipbuild.com/ship.aspx?pklujyukkpp4JsCcXanmkhTk8Pl4EN, https://www.shipvault.com/ships/502920, https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/502920</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -3167,7 +3167,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>https://www.worldoil.com/news/2026/7/10/adnoc-l-s-orders-four-lng-carriers-to-expand-global-shipping-fleet/, https://gasprocessingnews.com/news/2026/07/adnoc-ls-expands-lng-fleet-with-order-for-four-new-carriers/, http://www.chinashipbuild.com/ship.aspx?pklujyukkpp4JsCcXanmkhTk8Pl4EN, https://www.shipvault.com/ships/502921</t>
+          <t>https://www.worldoil.com/news/2026/7/10/adnoc-l-s-orders-four-lng-carriers-to-expand-global-shipping-fleet/, https://gasprocessingnews.com/news/2026/07/adnoc-ls-expands-lng-fleet-with-order-for-four-new-carriers/, http://www.chinashipbuild.com/ship.aspx?pklujyukkpp4JsCcXanmkhTk8Pl4EN, https://www.shipvault.com/ships/502921, https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/502921</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -3194,7 +3194,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>https://en.aletihad.ae/news/business/4687316/adnoc-l-s-orders-two-lng-carriers-for--444-million, https://www.seatrade-maritime.com/tankers/adnoc-l-s-adds-lng-carrier-pair-at-jiangnan-shipyard, https://www.shipvault.com/ships/503416</t>
+          <t>https://en.aletihad.ae/news/business/4687316/adnoc-l-s-orders-two-lng-carriers-for--444-million, https://www.seatrade-maritime.com/tankers/adnoc-l-s-adds-lng-carrier-pair-at-jiangnan-shipyard, https://www.shipvault.com/ships/503416, https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/503416</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -3221,7 +3221,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>https://en.aletihad.ae/news/business/4687316/adnoc-l-s-orders-two-lng-carriers-for--444-million, https://www.seatrade-maritime.com/tankers/adnoc-l-s-adds-lng-carrier-pair-at-jiangnan-shipyard, https://www.shipvault.com/ships/503417</t>
+          <t>https://en.aletihad.ae/news/business/4687316/adnoc-l-s-orders-two-lng-carriers-for--444-million, https://www.seatrade-maritime.com/tankers/adnoc-l-s-adds-lng-carrier-pair-at-jiangnan-shipyard, https://www.shipvault.com/ships/503417, https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/503417</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">

</xml_diff>

<commit_message>
discovery batch: drop unsourced vessel type on dynagas/tsakos rows; builder refuses values with no ref
</commit_message>
<xml_diff>
--- a/batches/2026-09-17_0431ET_discovery_since_jun_2026/lng_carrier_candidate_vessels.xlsx
+++ b/batches/2026-09-17_0431ET_discovery_since_jun_2026/lng_carrier_candidate_vessels.xlsx
@@ -604,7 +604,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX13"/>
+  <dimension ref="A1:BA13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -650,13 +650,16 @@
     <col width="15" customWidth="1" min="41" max="41"/>
     <col width="50" customWidth="1" min="42" max="42"/>
     <col width="15" customWidth="1" min="43" max="43"/>
-    <col width="25" customWidth="1" min="44" max="44"/>
+    <col width="15" customWidth="1" min="44" max="44"/>
     <col width="50" customWidth="1" min="45" max="45"/>
     <col width="15" customWidth="1" min="46" max="46"/>
-    <col width="50" customWidth="1" min="47" max="47"/>
-    <col width="15" customWidth="1" min="48" max="48"/>
+    <col width="25" customWidth="1" min="47" max="47"/>
+    <col width="50" customWidth="1" min="48" max="48"/>
     <col width="15" customWidth="1" min="49" max="49"/>
     <col width="50" customWidth="1" min="50" max="50"/>
+    <col width="15" customWidth="1" min="51" max="51"/>
+    <col width="15" customWidth="1" min="52" max="52"/>
+    <col width="50" customWidth="1" min="53" max="53"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -872,40 +875,55 @@
       </c>
       <c r="AQ1" s="3" t="inlineStr">
         <is>
+          <t>Delivery delayed</t>
+        </is>
+      </c>
+      <c r="AR1" s="3" t="inlineStr">
+        <is>
+          <t>Previous delivery year(s)</t>
+        </is>
+      </c>
+      <c r="AS1" s="3" t="inlineStr">
+        <is>
+          <t>Previous delivery year(s) [ref]</t>
+        </is>
+      </c>
+      <c r="AT1" s="3" t="inlineStr">
+        <is>
           <t>[Original source]</t>
         </is>
       </c>
-      <c r="AR1" s="3" t="inlineStr">
+      <c r="AU1" s="3" t="inlineStr">
         <is>
           <t>Operator/charterer</t>
         </is>
       </c>
-      <c r="AS1" s="3" t="inlineStr">
+      <c r="AV1" s="3" t="inlineStr">
         <is>
           <t>Operator/charterer [ref]</t>
         </is>
       </c>
-      <c r="AT1" s="3" t="inlineStr">
+      <c r="AW1" s="3" t="inlineStr">
         <is>
           <t>Contract date</t>
         </is>
       </c>
-      <c r="AU1" s="3" t="inlineStr">
+      <c r="AX1" s="3" t="inlineStr">
         <is>
           <t>Contract date [ref]</t>
         </is>
       </c>
-      <c r="AV1" s="3" t="inlineStr">
+      <c r="AY1" s="3" t="inlineStr">
         <is>
           <t>Price</t>
         </is>
       </c>
-      <c r="AW1" s="3" t="inlineStr">
+      <c r="AZ1" s="3" t="inlineStr">
         <is>
           <t>Price currency</t>
         </is>
       </c>
-      <c r="AX1" s="3" t="inlineStr">
+      <c r="BA1" s="3" t="inlineStr">
         <is>
           <t>Price [ref]</t>
         </is>
@@ -929,7 +947,7 @@
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>Samsung Heavy disclosed (DART, Mon 14-Sep-2026) a contract with an unidentified 'Oceania-based' owner for four 200,000 cu m LNG carriers, delivery by September 2029, combined value reported as ~$1.01bn (en.sedaily) / ~$1.05bn (Splash247) - two independently-reported total-price figures in the same ballpark, so per-vessel price is NOT included here (no source states a clean per-vessel USD figure that would pass the literal value-corroboration gate; computed averages would be ~$250-262.5M but that is my arithmetic, not sourced text). Splash247 (citing Greek market/broker sources) identifies the owner as Dynagas (George Procopiou), noting this is 'a change of builder' for Dynagas's large-LNG programme (previously concentrated at HD Hyundai Heavy Industries) - same identification pattern used elsewhere in this backend for broker-attributed owners (e.g. Purus Marine, Celsius Tankers), so graded G on two independent sources agreeing on yard/count/date, with the owner attribution flagged as market-source (not an official Samsung/DART naming). Not in baseline: baseline's latest Samsung HI contract date is 08-Jun-2026 (unknown shipowner 2). Vessel type: 200,000 cbm doesn't cleanly match the q-flex/q-max controlled-vocab bands (~210k/~266k) so left as 'conventional'. Propulsion type not stated in sources - omitted.</t>
+          <t>Samsung Heavy disclosed (DART, Mon 14-Sep-2026) a contract with an unidentified 'Oceania-based' owner for four 200,000 cu m LNG carriers, delivery by September 2029, combined value reported as ~$1.01bn (en.sedaily) / ~$1.05bn (Splash247) - two independently-reported total-price figures in the same ballpark, so per-vessel price is NOT included here (no source states a clean per-vessel USD figure that would pass the literal value-corroboration gate; computed averages would be ~$250-262.5M but that is my arithmetic, not sourced text). Splash247 (citing Greek market/broker sources) identifies the owner as Dynagas (George Procopiou), noting this is 'a change of builder' for Dynagas's large-LNG programme (previously concentrated at HD Hyundai Heavy Industries) - same identification pattern used elsewhere in this backend for broker-attributed owners (e.g. Purus Marine, Celsius Tankers), so graded G on two independent sources agreeing on yard/count/date, with the owner attribution flagged as market-source (not an official Samsung/DART naming). Not in baseline: baseline's latest Samsung HI contract date is 08-Jun-2026 (unknown shipowner 2). Vessel type left blank: no source states it (the cited pages, LNG Prime, new-ships, JoongAng say 'LNG carrier', never 'conventional'), so it is not written without a ref (DF SOP §9 note, RF §4.13). Propulsion type not stated in sources - omitted.</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr"/>
@@ -1032,11 +1050,7 @@
       </c>
       <c r="AI2" s="2" t="inlineStr"/>
       <c r="AJ2" s="2" t="inlineStr"/>
-      <c r="AK2" s="5" t="inlineStr">
-        <is>
-          <t>conventional</t>
-        </is>
-      </c>
+      <c r="AK2" s="2" t="inlineStr"/>
       <c r="AL2" s="2" t="inlineStr"/>
       <c r="AM2" s="2" t="inlineStr"/>
       <c r="AN2" s="2" t="inlineStr"/>
@@ -1053,19 +1067,22 @@
       <c r="AQ2" s="2" t="inlineStr"/>
       <c r="AR2" s="2" t="inlineStr"/>
       <c r="AS2" s="2" t="inlineStr"/>
-      <c r="AT2" s="5" t="inlineStr">
+      <c r="AT2" s="2" t="inlineStr"/>
+      <c r="AU2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AW2" s="5" t="inlineStr">
         <is>
           <t>14-Sep-2026</t>
         </is>
       </c>
-      <c r="AU2" s="5" t="inlineStr">
+      <c r="AX2" s="5" t="inlineStr">
         <is>
           <t>https://en.sedaily.com/finance/2026/09/14/samsung-heavy-wins-1b-order-for-four-lng-carriers</t>
         </is>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
-      <c r="AW2" s="2" t="inlineStr"/>
-      <c r="AX2" s="2" t="inlineStr"/>
+      <c r="AY2" s="2" t="inlineStr"/>
+      <c r="AZ2" s="2" t="inlineStr"/>
+      <c r="BA2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
@@ -1085,7 +1102,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>Samsung Heavy disclosed (DART, Mon 14-Sep-2026) a contract with an unidentified 'Oceania-based' owner for four 200,000 cu m LNG carriers, delivery by September 2029, combined value reported as ~$1.01bn (en.sedaily) / ~$1.05bn (Splash247) - two independently-reported total-price figures in the same ballpark, so per-vessel price is NOT included here (no source states a clean per-vessel USD figure that would pass the literal value-corroboration gate; computed averages would be ~$250-262.5M but that is my arithmetic, not sourced text). Splash247 (citing Greek market/broker sources) identifies the owner as Dynagas (George Procopiou), noting this is 'a change of builder' for Dynagas's large-LNG programme (previously concentrated at HD Hyundai Heavy Industries) - same identification pattern used elsewhere in this backend for broker-attributed owners (e.g. Purus Marine, Celsius Tankers), so graded G on two independent sources agreeing on yard/count/date, with the owner attribution flagged as market-source (not an official Samsung/DART naming). Not in baseline: baseline's latest Samsung HI contract date is 08-Jun-2026 (unknown shipowner 2). Vessel type: 200,000 cbm doesn't cleanly match the q-flex/q-max controlled-vocab bands (~210k/~266k) so left as 'conventional'. Propulsion type not stated in sources - omitted.</t>
+          <t>Samsung Heavy disclosed (DART, Mon 14-Sep-2026) a contract with an unidentified 'Oceania-based' owner for four 200,000 cu m LNG carriers, delivery by September 2029, combined value reported as ~$1.01bn (en.sedaily) / ~$1.05bn (Splash247) - two independently-reported total-price figures in the same ballpark, so per-vessel price is NOT included here (no source states a clean per-vessel USD figure that would pass the literal value-corroboration gate; computed averages would be ~$250-262.5M but that is my arithmetic, not sourced text). Splash247 (citing Greek market/broker sources) identifies the owner as Dynagas (George Procopiou), noting this is 'a change of builder' for Dynagas's large-LNG programme (previously concentrated at HD Hyundai Heavy Industries) - same identification pattern used elsewhere in this backend for broker-attributed owners (e.g. Purus Marine, Celsius Tankers), so graded G on two independent sources agreeing on yard/count/date, with the owner attribution flagged as market-source (not an official Samsung/DART naming). Not in baseline: baseline's latest Samsung HI contract date is 08-Jun-2026 (unknown shipowner 2). Vessel type left blank: no source states it (the cited pages, LNG Prime, new-ships, JoongAng say 'LNG carrier', never 'conventional'), so it is not written without a ref (DF SOP §9 note, RF §4.13). Propulsion type not stated in sources - omitted.</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr"/>
@@ -1188,11 +1205,7 @@
       </c>
       <c r="AI3" s="2" t="inlineStr"/>
       <c r="AJ3" s="2" t="inlineStr"/>
-      <c r="AK3" s="5" t="inlineStr">
-        <is>
-          <t>conventional</t>
-        </is>
-      </c>
+      <c r="AK3" s="2" t="inlineStr"/>
       <c r="AL3" s="2" t="inlineStr"/>
       <c r="AM3" s="2" t="inlineStr"/>
       <c r="AN3" s="2" t="inlineStr"/>
@@ -1209,19 +1222,22 @@
       <c r="AQ3" s="2" t="inlineStr"/>
       <c r="AR3" s="2" t="inlineStr"/>
       <c r="AS3" s="2" t="inlineStr"/>
-      <c r="AT3" s="5" t="inlineStr">
+      <c r="AT3" s="2" t="inlineStr"/>
+      <c r="AU3" s="2" t="inlineStr"/>
+      <c r="AV3" s="2" t="inlineStr"/>
+      <c r="AW3" s="5" t="inlineStr">
         <is>
           <t>14-Sep-2026</t>
         </is>
       </c>
-      <c r="AU3" s="5" t="inlineStr">
+      <c r="AX3" s="5" t="inlineStr">
         <is>
           <t>https://en.sedaily.com/finance/2026/09/14/samsung-heavy-wins-1b-order-for-four-lng-carriers</t>
         </is>
       </c>
-      <c r="AV3" s="2" t="inlineStr"/>
-      <c r="AW3" s="2" t="inlineStr"/>
-      <c r="AX3" s="2" t="inlineStr"/>
+      <c r="AY3" s="2" t="inlineStr"/>
+      <c r="AZ3" s="2" t="inlineStr"/>
+      <c r="BA3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
@@ -1241,7 +1257,7 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Samsung Heavy disclosed (DART, Mon 14-Sep-2026) a contract with an unidentified 'Oceania-based' owner for four 200,000 cu m LNG carriers, delivery by September 2029, combined value reported as ~$1.01bn (en.sedaily) / ~$1.05bn (Splash247) - two independently-reported total-price figures in the same ballpark, so per-vessel price is NOT included here (no source states a clean per-vessel USD figure that would pass the literal value-corroboration gate; computed averages would be ~$250-262.5M but that is my arithmetic, not sourced text). Splash247 (citing Greek market/broker sources) identifies the owner as Dynagas (George Procopiou), noting this is 'a change of builder' for Dynagas's large-LNG programme (previously concentrated at HD Hyundai Heavy Industries) - same identification pattern used elsewhere in this backend for broker-attributed owners (e.g. Purus Marine, Celsius Tankers), so graded G on two independent sources agreeing on yard/count/date, with the owner attribution flagged as market-source (not an official Samsung/DART naming). Not in baseline: baseline's latest Samsung HI contract date is 08-Jun-2026 (unknown shipowner 2). Vessel type: 200,000 cbm doesn't cleanly match the q-flex/q-max controlled-vocab bands (~210k/~266k) so left as 'conventional'. Propulsion type not stated in sources - omitted.</t>
+          <t>Samsung Heavy disclosed (DART, Mon 14-Sep-2026) a contract with an unidentified 'Oceania-based' owner for four 200,000 cu m LNG carriers, delivery by September 2029, combined value reported as ~$1.01bn (en.sedaily) / ~$1.05bn (Splash247) - two independently-reported total-price figures in the same ballpark, so per-vessel price is NOT included here (no source states a clean per-vessel USD figure that would pass the literal value-corroboration gate; computed averages would be ~$250-262.5M but that is my arithmetic, not sourced text). Splash247 (citing Greek market/broker sources) identifies the owner as Dynagas (George Procopiou), noting this is 'a change of builder' for Dynagas's large-LNG programme (previously concentrated at HD Hyundai Heavy Industries) - same identification pattern used elsewhere in this backend for broker-attributed owners (e.g. Purus Marine, Celsius Tankers), so graded G on two independent sources agreeing on yard/count/date, with the owner attribution flagged as market-source (not an official Samsung/DART naming). Not in baseline: baseline's latest Samsung HI contract date is 08-Jun-2026 (unknown shipowner 2). Vessel type left blank: no source states it (the cited pages, LNG Prime, new-ships, JoongAng say 'LNG carrier', never 'conventional'), so it is not written without a ref (DF SOP §9 note, RF §4.13). Propulsion type not stated in sources - omitted.</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr"/>
@@ -1344,11 +1360,7 @@
       </c>
       <c r="AI4" s="2" t="inlineStr"/>
       <c r="AJ4" s="2" t="inlineStr"/>
-      <c r="AK4" s="5" t="inlineStr">
-        <is>
-          <t>conventional</t>
-        </is>
-      </c>
+      <c r="AK4" s="2" t="inlineStr"/>
       <c r="AL4" s="2" t="inlineStr"/>
       <c r="AM4" s="2" t="inlineStr"/>
       <c r="AN4" s="2" t="inlineStr"/>
@@ -1365,19 +1377,22 @@
       <c r="AQ4" s="2" t="inlineStr"/>
       <c r="AR4" s="2" t="inlineStr"/>
       <c r="AS4" s="2" t="inlineStr"/>
-      <c r="AT4" s="5" t="inlineStr">
+      <c r="AT4" s="2" t="inlineStr"/>
+      <c r="AU4" s="2" t="inlineStr"/>
+      <c r="AV4" s="2" t="inlineStr"/>
+      <c r="AW4" s="5" t="inlineStr">
         <is>
           <t>14-Sep-2026</t>
         </is>
       </c>
-      <c r="AU4" s="5" t="inlineStr">
+      <c r="AX4" s="5" t="inlineStr">
         <is>
           <t>https://en.sedaily.com/finance/2026/09/14/samsung-heavy-wins-1b-order-for-four-lng-carriers</t>
         </is>
       </c>
-      <c r="AV4" s="2" t="inlineStr"/>
-      <c r="AW4" s="2" t="inlineStr"/>
-      <c r="AX4" s="2" t="inlineStr"/>
+      <c r="AY4" s="2" t="inlineStr"/>
+      <c r="AZ4" s="2" t="inlineStr"/>
+      <c r="BA4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -1397,7 +1412,7 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Samsung Heavy disclosed (DART, Mon 14-Sep-2026) a contract with an unidentified 'Oceania-based' owner for four 200,000 cu m LNG carriers, delivery by September 2029, combined value reported as ~$1.01bn (en.sedaily) / ~$1.05bn (Splash247) - two independently-reported total-price figures in the same ballpark, so per-vessel price is NOT included here (no source states a clean per-vessel USD figure that would pass the literal value-corroboration gate; computed averages would be ~$250-262.5M but that is my arithmetic, not sourced text). Splash247 (citing Greek market/broker sources) identifies the owner as Dynagas (George Procopiou), noting this is 'a change of builder' for Dynagas's large-LNG programme (previously concentrated at HD Hyundai Heavy Industries) - same identification pattern used elsewhere in this backend for broker-attributed owners (e.g. Purus Marine, Celsius Tankers), so graded G on two independent sources agreeing on yard/count/date, with the owner attribution flagged as market-source (not an official Samsung/DART naming). Not in baseline: baseline's latest Samsung HI contract date is 08-Jun-2026 (unknown shipowner 2). Vessel type: 200,000 cbm doesn't cleanly match the q-flex/q-max controlled-vocab bands (~210k/~266k) so left as 'conventional'. Propulsion type not stated in sources - omitted.</t>
+          <t>Samsung Heavy disclosed (DART, Mon 14-Sep-2026) a contract with an unidentified 'Oceania-based' owner for four 200,000 cu m LNG carriers, delivery by September 2029, combined value reported as ~$1.01bn (en.sedaily) / ~$1.05bn (Splash247) - two independently-reported total-price figures in the same ballpark, so per-vessel price is NOT included here (no source states a clean per-vessel USD figure that would pass the literal value-corroboration gate; computed averages would be ~$250-262.5M but that is my arithmetic, not sourced text). Splash247 (citing Greek market/broker sources) identifies the owner as Dynagas (George Procopiou), noting this is 'a change of builder' for Dynagas's large-LNG programme (previously concentrated at HD Hyundai Heavy Industries) - same identification pattern used elsewhere in this backend for broker-attributed owners (e.g. Purus Marine, Celsius Tankers), so graded G on two independent sources agreeing on yard/count/date, with the owner attribution flagged as market-source (not an official Samsung/DART naming). Not in baseline: baseline's latest Samsung HI contract date is 08-Jun-2026 (unknown shipowner 2). Vessel type left blank: no source states it (the cited pages, LNG Prime, new-ships, JoongAng say 'LNG carrier', never 'conventional'), so it is not written without a ref (DF SOP §9 note, RF §4.13). Propulsion type not stated in sources - omitted.</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr"/>
@@ -1500,11 +1515,7 @@
       </c>
       <c r="AI5" s="2" t="inlineStr"/>
       <c r="AJ5" s="2" t="inlineStr"/>
-      <c r="AK5" s="5" t="inlineStr">
-        <is>
-          <t>conventional</t>
-        </is>
-      </c>
+      <c r="AK5" s="2" t="inlineStr"/>
       <c r="AL5" s="2" t="inlineStr"/>
       <c r="AM5" s="2" t="inlineStr"/>
       <c r="AN5" s="2" t="inlineStr"/>
@@ -1521,19 +1532,22 @@
       <c r="AQ5" s="2" t="inlineStr"/>
       <c r="AR5" s="2" t="inlineStr"/>
       <c r="AS5" s="2" t="inlineStr"/>
-      <c r="AT5" s="5" t="inlineStr">
+      <c r="AT5" s="2" t="inlineStr"/>
+      <c r="AU5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AW5" s="5" t="inlineStr">
         <is>
           <t>14-Sep-2026</t>
         </is>
       </c>
-      <c r="AU5" s="5" t="inlineStr">
+      <c r="AX5" s="5" t="inlineStr">
         <is>
           <t>https://en.sedaily.com/finance/2026/09/14/samsung-heavy-wins-1b-order-for-four-lng-carriers</t>
         </is>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
-      <c r="AW5" s="2" t="inlineStr"/>
-      <c r="AX5" s="2" t="inlineStr"/>
+      <c r="AY5" s="2" t="inlineStr"/>
+      <c r="AZ5" s="2" t="inlineStr"/>
+      <c r="BA5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -1553,7 +1567,7 @@
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>TEN Ltd's own press release (GlobeNewswire, 01-Jul-2026) announces a SECOND LNG carrier order at HD Hyundai Heavy Industries, explicitly described as 'an option attached to the order announced in February' (i.e. an exercised option on the Feb-2026 contract already in the backend as HD Hyundai HI (HHI) Ulsan 3643 / Tsakos, 25-Feb-2026, 174000cbm, 2028). This is a genuinely new hull, in scope per the task brief ('exercised option'). Riviera corroborates: price ~US$254M, delivery by January 2029 (Q1 2029), yard HD Hyundai Heavy Industries. This July disclosure lines up with HD Korea Shipbuilding's same-day (30-Jun-2026 signing / reported 01-Jul-2026) 392.2 billion won LNG-carrier disclosure (~$253M at the same day's exchange rate implied by the $570.7M/885bn-won combined figure) - consistent with this being that vessel. Capacity: not explicitly re-stated as '174,000' in the confirmed-order articles (Riviera/GlobeNewswire), so Capacity is left OUT of row_data per the literal-value rule, even though it is highly likely 174,000cbm given TEN's existing 174,000cbm fleet and prior contract - noting this as a probable-but-unsourced fact rather than guessing it into a cited cell. Not in baseline: baseline's only Tsakos row is the single 25-Feb-2026 vessel; this is an additional/second one.</t>
+          <t>TEN Ltd's own press release (GlobeNewswire, 01-Jul-2026) announces a SECOND LNG carrier order at HD Hyundai Heavy Industries, explicitly described as 'an option attached to the order announced in February' (i.e. an exercised option on the Feb-2026 contract already in the backend as HD Hyundai HI (HHI) Ulsan 3643 / Tsakos, 25-Feb-2026, 174000cbm, 2028). This is a genuinely new hull, in scope per the task brief ('exercised option'). Riviera corroborates: price ~US$254M, delivery by January 2029 (Q1 2029), yard HD Hyundai Heavy Industries. This July disclosure lines up with HD Korea Shipbuilding's same-day (30-Jun-2026 signing / reported 01-Jul-2026) 392.2 billion won LNG-carrier disclosure (~$253M at the same day's exchange rate implied by the $570.7M/885bn-won combined figure) - consistent with this being that vessel. Capacity: not explicitly re-stated as '174,000' in the confirmed-order articles (Riviera/GlobeNewswire), so Capacity is left OUT of row_data per the literal-value rule, even though it is highly likely 174,000cbm given TEN's existing 174,000cbm fleet and prior contract - noting this as a probable-but-unsourced fact rather than guessing it into a cited cell. Not in baseline: baseline's only Tsakos row is the single 25-Feb-2026 vessel; this is an additional/second one. Vessel type left blank: no source states 'conventional' for this hull (GlobeNewswire, Riviera, Splash247 checked).</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr"/>
@@ -1644,11 +1658,7 @@
       <c r="AH6" s="2" t="inlineStr"/>
       <c r="AI6" s="2" t="inlineStr"/>
       <c r="AJ6" s="2" t="inlineStr"/>
-      <c r="AK6" s="7" t="inlineStr">
-        <is>
-          <t>conventional</t>
-        </is>
-      </c>
+      <c r="AK6" s="2" t="inlineStr"/>
       <c r="AL6" s="2" t="inlineStr"/>
       <c r="AM6" s="2" t="inlineStr"/>
       <c r="AN6" s="2" t="inlineStr"/>
@@ -1663,37 +1673,40 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="inlineStr"/>
-      <c r="AR6" s="7" t="inlineStr">
+      <c r="AR6" s="2" t="inlineStr"/>
+      <c r="AS6" s="2" t="inlineStr"/>
+      <c r="AT6" s="2" t="inlineStr"/>
+      <c r="AU6" s="7" t="inlineStr">
         <is>
           <t>Tsakos</t>
         </is>
       </c>
-      <c r="AS6" s="7" t="inlineStr">
+      <c r="AV6" s="7" t="inlineStr">
         <is>
           <t>https://www.globenewswire.com/news-release/2026/07/01/3320982/0/en/TEN-Ltd-Announces-Second-LNG-Carrier-Order-in-Hyundai-Heavy-Industries.html</t>
         </is>
       </c>
-      <c r="AT6" s="7" t="inlineStr">
+      <c r="AW6" s="7" t="inlineStr">
         <is>
           <t>01-Jul-2026</t>
         </is>
       </c>
-      <c r="AU6" s="7" t="inlineStr">
+      <c r="AX6" s="7" t="inlineStr">
         <is>
           <t>https://www.globenewswire.com/news-release/2026/07/01/3320982/0/en/TEN-Ltd-Announces-Second-LNG-Carrier-Order-in-Hyundai-Heavy-Industries.html</t>
         </is>
       </c>
-      <c r="AV6" s="7" t="inlineStr">
+      <c r="AY6" s="7" t="inlineStr">
         <is>
           <t>254000000</t>
         </is>
       </c>
-      <c r="AW6" s="7" t="inlineStr">
+      <c r="AZ6" s="7" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="AX6" s="7" t="inlineStr">
+      <c r="BA6" s="7" t="inlineStr">
         <is>
           <t>https://www.rivieramm.com/news-content-hub/tsakos-orders-second-lng-carrier-in-korea-lifting-orderbook-to-20-vessels-89259</t>
         </is>
@@ -1829,19 +1842,22 @@
       <c r="AQ7" s="2" t="inlineStr"/>
       <c r="AR7" s="2" t="inlineStr"/>
       <c r="AS7" s="2" t="inlineStr"/>
-      <c r="AT7" s="5" t="inlineStr">
+      <c r="AT7" s="2" t="inlineStr"/>
+      <c r="AU7" s="2" t="inlineStr"/>
+      <c r="AV7" s="2" t="inlineStr"/>
+      <c r="AW7" s="5" t="inlineStr">
         <is>
           <t>30-Jun-2026</t>
         </is>
       </c>
-      <c r="AU7" s="5" t="inlineStr">
+      <c r="AX7" s="5" t="inlineStr">
         <is>
           <t>https://en.sedaily.com/finance/2026/07/01/hd-korea-shipbuilding-wins-885-billion-won-order-for-two</t>
         </is>
       </c>
-      <c r="AV7" s="2" t="inlineStr"/>
-      <c r="AW7" s="2" t="inlineStr"/>
-      <c r="AX7" s="2" t="inlineStr"/>
+      <c r="AY7" s="2" t="inlineStr"/>
+      <c r="AZ7" s="2" t="inlineStr"/>
+      <c r="BA7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
@@ -1997,19 +2013,22 @@
       <c r="AQ8" s="2" t="inlineStr"/>
       <c r="AR8" s="2" t="inlineStr"/>
       <c r="AS8" s="2" t="inlineStr"/>
-      <c r="AT8" s="7" t="inlineStr">
+      <c r="AT8" s="2" t="inlineStr"/>
+      <c r="AU8" s="2" t="inlineStr"/>
+      <c r="AV8" s="2" t="inlineStr"/>
+      <c r="AW8" s="7" t="inlineStr">
         <is>
           <t>10-Jul-2026</t>
         </is>
       </c>
-      <c r="AU8" s="7" t="inlineStr">
+      <c r="AX8" s="7" t="inlineStr">
         <is>
           <t>https://www.worldoil.com/news/2026/7/10/adnoc-l-s-orders-four-lng-carriers-to-expand-global-shipping-fleet/</t>
         </is>
       </c>
-      <c r="AV8" s="2" t="inlineStr"/>
-      <c r="AW8" s="2" t="inlineStr"/>
-      <c r="AX8" s="2" t="inlineStr"/>
+      <c r="AY8" s="2" t="inlineStr"/>
+      <c r="AZ8" s="2" t="inlineStr"/>
+      <c r="BA8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
@@ -2165,19 +2184,22 @@
       <c r="AQ9" s="2" t="inlineStr"/>
       <c r="AR9" s="2" t="inlineStr"/>
       <c r="AS9" s="2" t="inlineStr"/>
-      <c r="AT9" s="7" t="inlineStr">
+      <c r="AT9" s="2" t="inlineStr"/>
+      <c r="AU9" s="2" t="inlineStr"/>
+      <c r="AV9" s="2" t="inlineStr"/>
+      <c r="AW9" s="7" t="inlineStr">
         <is>
           <t>10-Jul-2026</t>
         </is>
       </c>
-      <c r="AU9" s="7" t="inlineStr">
+      <c r="AX9" s="7" t="inlineStr">
         <is>
           <t>https://www.worldoil.com/news/2026/7/10/adnoc-l-s-orders-four-lng-carriers-to-expand-global-shipping-fleet/</t>
         </is>
       </c>
-      <c r="AV9" s="2" t="inlineStr"/>
-      <c r="AW9" s="2" t="inlineStr"/>
-      <c r="AX9" s="2" t="inlineStr"/>
+      <c r="AY9" s="2" t="inlineStr"/>
+      <c r="AZ9" s="2" t="inlineStr"/>
+      <c r="BA9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
@@ -2333,19 +2355,22 @@
       <c r="AQ10" s="2" t="inlineStr"/>
       <c r="AR10" s="2" t="inlineStr"/>
       <c r="AS10" s="2" t="inlineStr"/>
-      <c r="AT10" s="7" t="inlineStr">
+      <c r="AT10" s="2" t="inlineStr"/>
+      <c r="AU10" s="2" t="inlineStr"/>
+      <c r="AV10" s="2" t="inlineStr"/>
+      <c r="AW10" s="7" t="inlineStr">
         <is>
           <t>10-Jul-2026</t>
         </is>
       </c>
-      <c r="AU10" s="7" t="inlineStr">
+      <c r="AX10" s="7" t="inlineStr">
         <is>
           <t>https://www.worldoil.com/news/2026/7/10/adnoc-l-s-orders-four-lng-carriers-to-expand-global-shipping-fleet/</t>
         </is>
       </c>
-      <c r="AV10" s="2" t="inlineStr"/>
-      <c r="AW10" s="2" t="inlineStr"/>
-      <c r="AX10" s="2" t="inlineStr"/>
+      <c r="AY10" s="2" t="inlineStr"/>
+      <c r="AZ10" s="2" t="inlineStr"/>
+      <c r="BA10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
@@ -2501,19 +2526,22 @@
       <c r="AQ11" s="2" t="inlineStr"/>
       <c r="AR11" s="2" t="inlineStr"/>
       <c r="AS11" s="2" t="inlineStr"/>
-      <c r="AT11" s="7" t="inlineStr">
+      <c r="AT11" s="2" t="inlineStr"/>
+      <c r="AU11" s="2" t="inlineStr"/>
+      <c r="AV11" s="2" t="inlineStr"/>
+      <c r="AW11" s="7" t="inlineStr">
         <is>
           <t>10-Jul-2026</t>
         </is>
       </c>
-      <c r="AU11" s="7" t="inlineStr">
+      <c r="AX11" s="7" t="inlineStr">
         <is>
           <t>https://www.worldoil.com/news/2026/7/10/adnoc-l-s-orders-four-lng-carriers-to-expand-global-shipping-fleet/</t>
         </is>
       </c>
-      <c r="AV11" s="2" t="inlineStr"/>
-      <c r="AW11" s="2" t="inlineStr"/>
-      <c r="AX11" s="2" t="inlineStr"/>
+      <c r="AY11" s="2" t="inlineStr"/>
+      <c r="AZ11" s="2" t="inlineStr"/>
+      <c r="BA11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
@@ -2669,19 +2697,22 @@
       <c r="AQ12" s="2" t="inlineStr"/>
       <c r="AR12" s="2" t="inlineStr"/>
       <c r="AS12" s="2" t="inlineStr"/>
-      <c r="AT12" s="7" t="inlineStr">
+      <c r="AT12" s="2" t="inlineStr"/>
+      <c r="AU12" s="2" t="inlineStr"/>
+      <c r="AV12" s="2" t="inlineStr"/>
+      <c r="AW12" s="7" t="inlineStr">
         <is>
           <t>25-Aug-2026</t>
         </is>
       </c>
-      <c r="AU12" s="7" t="inlineStr">
+      <c r="AX12" s="7" t="inlineStr">
         <is>
           <t>https://en.aletihad.ae/news/business/4687316/adnoc-l-s-orders-two-lng-carriers-for--444-million</t>
         </is>
       </c>
-      <c r="AV12" s="2" t="inlineStr"/>
-      <c r="AW12" s="2" t="inlineStr"/>
-      <c r="AX12" s="2" t="inlineStr"/>
+      <c r="AY12" s="2" t="inlineStr"/>
+      <c r="AZ12" s="2" t="inlineStr"/>
+      <c r="BA12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
@@ -2837,19 +2868,22 @@
       <c r="AQ13" s="2" t="inlineStr"/>
       <c r="AR13" s="2" t="inlineStr"/>
       <c r="AS13" s="2" t="inlineStr"/>
-      <c r="AT13" s="7" t="inlineStr">
+      <c r="AT13" s="2" t="inlineStr"/>
+      <c r="AU13" s="2" t="inlineStr"/>
+      <c r="AV13" s="2" t="inlineStr"/>
+      <c r="AW13" s="7" t="inlineStr">
         <is>
           <t>25-Aug-2026</t>
         </is>
       </c>
-      <c r="AU13" s="7" t="inlineStr">
+      <c r="AX13" s="7" t="inlineStr">
         <is>
           <t>https://en.aletihad.ae/news/business/4687316/adnoc-l-s-orders-two-lng-carriers-for--444-million</t>
         </is>
       </c>
-      <c r="AV13" s="2" t="inlineStr"/>
-      <c r="AW13" s="2" t="inlineStr"/>
-      <c r="AX13" s="2" t="inlineStr"/>
+      <c r="AY13" s="2" t="inlineStr"/>
+      <c r="AZ13" s="2" t="inlineStr"/>
+      <c r="BA13" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2929,7 +2963,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Samsung Heavy disclosed (DART, Mon 14-Sep-2026) a contract with an unidentified 'Oceania-based' owner for four 200,000 cu m LNG carriers, delivery by September 2029, combined value reported as ~$1.01bn (en.sedaily) / ~$1.05bn (Splash247) - two independently-reported total-price figures in the same ballpark, so per-vessel price is NOT included here (no source states a clean per-vessel USD figure that would pass the literal value-corroboration gate; computed averages would be ~$250-262.5M but that is my arithmetic, not sourced text). Splash247 (citing Greek market/broker sources) identifies the owner as Dynagas (George Procopiou), noting this is 'a change of builder' for Dynagas's large-LNG programme (previously concentrated at HD Hyundai Heavy Industries) - same identification pattern used elsewhere in this backend for broker-attributed owners (e.g. Purus Marine, Celsius Tankers), so graded G on two independent sources agreeing on yard/count/date, with the owner attribution flagged as market-source (not an official Samsung/DART naming). Not in baseline: baseline's latest Samsung HI contract date is 08-Jun-2026 (unknown shipowner 2). Vessel type: 200,000 cbm doesn't cleanly match the q-flex/q-max controlled-vocab bands (~210k/~266k) so left as 'conventional'. Propulsion type not stated in sources - omitted.</t>
+          <t>Samsung Heavy disclosed (DART, Mon 14-Sep-2026) a contract with an unidentified 'Oceania-based' owner for four 200,000 cu m LNG carriers, delivery by September 2029, combined value reported as ~$1.01bn (en.sedaily) / ~$1.05bn (Splash247) - two independently-reported total-price figures in the same ballpark, so per-vessel price is NOT included here (no source states a clean per-vessel USD figure that would pass the literal value-corroboration gate; computed averages would be ~$250-262.5M but that is my arithmetic, not sourced text). Splash247 (citing Greek market/broker sources) identifies the owner as Dynagas (George Procopiou), noting this is 'a change of builder' for Dynagas's large-LNG programme (previously concentrated at HD Hyundai Heavy Industries) - same identification pattern used elsewhere in this backend for broker-attributed owners (e.g. Purus Marine, Celsius Tankers), so graded G on two independent sources agreeing on yard/count/date, with the owner attribution flagged as market-source (not an official Samsung/DART naming). Not in baseline: baseline's latest Samsung HI contract date is 08-Jun-2026 (unknown shipowner 2). Vessel type left blank: no source states it (the cited pages, LNG Prime, new-ships, JoongAng say 'LNG carrier', never 'conventional'), so it is not written without a ref (DF SOP §9 note, RF §4.13). Propulsion type not stated in sources - omitted.</t>
         </is>
       </c>
     </row>
@@ -2956,7 +2990,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Samsung Heavy disclosed (DART, Mon 14-Sep-2026) a contract with an unidentified 'Oceania-based' owner for four 200,000 cu m LNG carriers, delivery by September 2029, combined value reported as ~$1.01bn (en.sedaily) / ~$1.05bn (Splash247) - two independently-reported total-price figures in the same ballpark, so per-vessel price is NOT included here (no source states a clean per-vessel USD figure that would pass the literal value-corroboration gate; computed averages would be ~$250-262.5M but that is my arithmetic, not sourced text). Splash247 (citing Greek market/broker sources) identifies the owner as Dynagas (George Procopiou), noting this is 'a change of builder' for Dynagas's large-LNG programme (previously concentrated at HD Hyundai Heavy Industries) - same identification pattern used elsewhere in this backend for broker-attributed owners (e.g. Purus Marine, Celsius Tankers), so graded G on two independent sources agreeing on yard/count/date, with the owner attribution flagged as market-source (not an official Samsung/DART naming). Not in baseline: baseline's latest Samsung HI contract date is 08-Jun-2026 (unknown shipowner 2). Vessel type: 200,000 cbm doesn't cleanly match the q-flex/q-max controlled-vocab bands (~210k/~266k) so left as 'conventional'. Propulsion type not stated in sources - omitted.</t>
+          <t>Samsung Heavy disclosed (DART, Mon 14-Sep-2026) a contract with an unidentified 'Oceania-based' owner for four 200,000 cu m LNG carriers, delivery by September 2029, combined value reported as ~$1.01bn (en.sedaily) / ~$1.05bn (Splash247) - two independently-reported total-price figures in the same ballpark, so per-vessel price is NOT included here (no source states a clean per-vessel USD figure that would pass the literal value-corroboration gate; computed averages would be ~$250-262.5M but that is my arithmetic, not sourced text). Splash247 (citing Greek market/broker sources) identifies the owner as Dynagas (George Procopiou), noting this is 'a change of builder' for Dynagas's large-LNG programme (previously concentrated at HD Hyundai Heavy Industries) - same identification pattern used elsewhere in this backend for broker-attributed owners (e.g. Purus Marine, Celsius Tankers), so graded G on two independent sources agreeing on yard/count/date, with the owner attribution flagged as market-source (not an official Samsung/DART naming). Not in baseline: baseline's latest Samsung HI contract date is 08-Jun-2026 (unknown shipowner 2). Vessel type left blank: no source states it (the cited pages, LNG Prime, new-ships, JoongAng say 'LNG carrier', never 'conventional'), so it is not written without a ref (DF SOP §9 note, RF §4.13). Propulsion type not stated in sources - omitted.</t>
         </is>
       </c>
     </row>
@@ -2983,7 +3017,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Samsung Heavy disclosed (DART, Mon 14-Sep-2026) a contract with an unidentified 'Oceania-based' owner for four 200,000 cu m LNG carriers, delivery by September 2029, combined value reported as ~$1.01bn (en.sedaily) / ~$1.05bn (Splash247) - two independently-reported total-price figures in the same ballpark, so per-vessel price is NOT included here (no source states a clean per-vessel USD figure that would pass the literal value-corroboration gate; computed averages would be ~$250-262.5M but that is my arithmetic, not sourced text). Splash247 (citing Greek market/broker sources) identifies the owner as Dynagas (George Procopiou), noting this is 'a change of builder' for Dynagas's large-LNG programme (previously concentrated at HD Hyundai Heavy Industries) - same identification pattern used elsewhere in this backend for broker-attributed owners (e.g. Purus Marine, Celsius Tankers), so graded G on two independent sources agreeing on yard/count/date, with the owner attribution flagged as market-source (not an official Samsung/DART naming). Not in baseline: baseline's latest Samsung HI contract date is 08-Jun-2026 (unknown shipowner 2). Vessel type: 200,000 cbm doesn't cleanly match the q-flex/q-max controlled-vocab bands (~210k/~266k) so left as 'conventional'. Propulsion type not stated in sources - omitted.</t>
+          <t>Samsung Heavy disclosed (DART, Mon 14-Sep-2026) a contract with an unidentified 'Oceania-based' owner for four 200,000 cu m LNG carriers, delivery by September 2029, combined value reported as ~$1.01bn (en.sedaily) / ~$1.05bn (Splash247) - two independently-reported total-price figures in the same ballpark, so per-vessel price is NOT included here (no source states a clean per-vessel USD figure that would pass the literal value-corroboration gate; computed averages would be ~$250-262.5M but that is my arithmetic, not sourced text). Splash247 (citing Greek market/broker sources) identifies the owner as Dynagas (George Procopiou), noting this is 'a change of builder' for Dynagas's large-LNG programme (previously concentrated at HD Hyundai Heavy Industries) - same identification pattern used elsewhere in this backend for broker-attributed owners (e.g. Purus Marine, Celsius Tankers), so graded G on two independent sources agreeing on yard/count/date, with the owner attribution flagged as market-source (not an official Samsung/DART naming). Not in baseline: baseline's latest Samsung HI contract date is 08-Jun-2026 (unknown shipowner 2). Vessel type left blank: no source states it (the cited pages, LNG Prime, new-ships, JoongAng say 'LNG carrier', never 'conventional'), so it is not written without a ref (DF SOP §9 note, RF §4.13). Propulsion type not stated in sources - omitted.</t>
         </is>
       </c>
     </row>
@@ -3010,7 +3044,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Samsung Heavy disclosed (DART, Mon 14-Sep-2026) a contract with an unidentified 'Oceania-based' owner for four 200,000 cu m LNG carriers, delivery by September 2029, combined value reported as ~$1.01bn (en.sedaily) / ~$1.05bn (Splash247) - two independently-reported total-price figures in the same ballpark, so per-vessel price is NOT included here (no source states a clean per-vessel USD figure that would pass the literal value-corroboration gate; computed averages would be ~$250-262.5M but that is my arithmetic, not sourced text). Splash247 (citing Greek market/broker sources) identifies the owner as Dynagas (George Procopiou), noting this is 'a change of builder' for Dynagas's large-LNG programme (previously concentrated at HD Hyundai Heavy Industries) - same identification pattern used elsewhere in this backend for broker-attributed owners (e.g. Purus Marine, Celsius Tankers), so graded G on two independent sources agreeing on yard/count/date, with the owner attribution flagged as market-source (not an official Samsung/DART naming). Not in baseline: baseline's latest Samsung HI contract date is 08-Jun-2026 (unknown shipowner 2). Vessel type: 200,000 cbm doesn't cleanly match the q-flex/q-max controlled-vocab bands (~210k/~266k) so left as 'conventional'. Propulsion type not stated in sources - omitted.</t>
+          <t>Samsung Heavy disclosed (DART, Mon 14-Sep-2026) a contract with an unidentified 'Oceania-based' owner for four 200,000 cu m LNG carriers, delivery by September 2029, combined value reported as ~$1.01bn (en.sedaily) / ~$1.05bn (Splash247) - two independently-reported total-price figures in the same ballpark, so per-vessel price is NOT included here (no source states a clean per-vessel USD figure that would pass the literal value-corroboration gate; computed averages would be ~$250-262.5M but that is my arithmetic, not sourced text). Splash247 (citing Greek market/broker sources) identifies the owner as Dynagas (George Procopiou), noting this is 'a change of builder' for Dynagas's large-LNG programme (previously concentrated at HD Hyundai Heavy Industries) - same identification pattern used elsewhere in this backend for broker-attributed owners (e.g. Purus Marine, Celsius Tankers), so graded G on two independent sources agreeing on yard/count/date, with the owner attribution flagged as market-source (not an official Samsung/DART naming). Not in baseline: baseline's latest Samsung HI contract date is 08-Jun-2026 (unknown shipowner 2). Vessel type left blank: no source states it (the cited pages, LNG Prime, new-ships, JoongAng say 'LNG carrier', never 'conventional'), so it is not written without a ref (DF SOP §9 note, RF §4.13). Propulsion type not stated in sources - omitted.</t>
         </is>
       </c>
     </row>
@@ -3037,7 +3071,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>TEN Ltd's own press release (GlobeNewswire, 01-Jul-2026) announces a SECOND LNG carrier order at HD Hyundai Heavy Industries, explicitly described as 'an option attached to the order announced in February' (i.e. an exercised option on the Feb-2026 contract already in the backend as HD Hyundai HI (HHI) Ulsan 3643 / Tsakos, 25-Feb-2026, 174000cbm, 2028). This is a genuinely new hull, in scope per the task brief ('exercised option'). Riviera corroborates: price ~US$254M, delivery by January 2029 (Q1 2029), yard HD Hyundai Heavy Industries. This July disclosure lines up with HD Korea Shipbuilding's same-day (30-Jun-2026 signing / reported 01-Jul-2026) 392.2 billion won LNG-carrier disclosure (~$253M at the same day's exchange rate implied by the $570.7M/885bn-won combined figure) - consistent with this being that vessel. Capacity: not explicitly re-stated as '174,000' in the confirmed-order articles (Riviera/GlobeNewswire), so Capacity is left OUT of row_data per the literal-value rule, even though it is highly likely 174,000cbm given TEN's existing 174,000cbm fleet and prior contract - noting this as a probable-but-unsourced fact rather than guessing it into a cited cell. Not in baseline: baseline's only Tsakos row is the single 25-Feb-2026 vessel; this is an additional/second one.</t>
+          <t>TEN Ltd's own press release (GlobeNewswire, 01-Jul-2026) announces a SECOND LNG carrier order at HD Hyundai Heavy Industries, explicitly described as 'an option attached to the order announced in February' (i.e. an exercised option on the Feb-2026 contract already in the backend as HD Hyundai HI (HHI) Ulsan 3643 / Tsakos, 25-Feb-2026, 174000cbm, 2028). This is a genuinely new hull, in scope per the task brief ('exercised option'). Riviera corroborates: price ~US$254M, delivery by January 2029 (Q1 2029), yard HD Hyundai Heavy Industries. This July disclosure lines up with HD Korea Shipbuilding's same-day (30-Jun-2026 signing / reported 01-Jul-2026) 392.2 billion won LNG-carrier disclosure (~$253M at the same day's exchange rate implied by the $570.7M/885bn-won combined figure) - consistent with this being that vessel. Capacity: not explicitly re-stated as '174,000' in the confirmed-order articles (Riviera/GlobeNewswire), so Capacity is left OUT of row_data per the literal-value rule, even though it is highly likely 174,000cbm given TEN's existing 174,000cbm fleet and prior contract - noting this as a probable-but-unsourced fact rather than guessing it into a cited cell. Not in baseline: baseline's only Tsakos row is the single 25-Feb-2026 vessel; this is an additional/second one. Vessel type left blank: no source states 'conventional' for this hull (GlobeNewswire, Riviera, Splash247 checked).</t>
         </is>
       </c>
     </row>

</xml_diff>